<commit_message>
Add missing functionality, unit tests, workbook test and clean-up files.
</commit_message>
<xml_diff>
--- a/tests/workbooktests/workbooks/extras/test_alias_repository.xlsx
+++ b/tests/workbooktests/workbooks/extras/test_alias_repository.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebastian\01_GitHub\sschlenkrich\QuantLibXlOil\tests\workbooktests\workbooks\extras\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\tests\workbooktests\workbooks\extras\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69B60D5-F571-42D9-A316-C6327320B5D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{667365C7-64FF-45F6-AAFB-37D7E1C3511D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{74A8DA6A-BC56-4206-BAAB-E5B423CC98C8}"/>
+    <workbookView xWindow="-120" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{74A8DA6A-BC56-4206-BAAB-E5B423CC98C8}"/>
   </bookViews>
   <sheets>
     <sheet name="Ibor Leg" sheetId="2" r:id="rId1"/>
@@ -21,17 +21,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -40,14 +29,14 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
   <futureMetadata name="XLDAPR" count="1">
     <bk>
       <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+        <ext xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray" uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
           <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
         </ext>
       </extLst>
@@ -125,7 +114,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -180,7 +169,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -513,13 +502,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73DF8D7F-06F7-4C65-A83C-66B48A78A848}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="22.109375" customWidth="1"/>
-    <col min="2" max="2" width="68.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.125" customWidth="1"/>
+    <col min="2" max="2" width="68.875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -527,7 +516,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -536,25 +525,25 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="str" cm="1">
-        <f t="array" ref="B4">_xll.qlFlatForward($B$2,0.03)</f>
+      <c r="B4" s="2" t="str">
+        <f>_xll.qlFlatForward($B$2,0.03,"actual365fixed")</f>
         <v>欣[test_alias_repository.xlsx]Ibor Leg!R4C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="2" t="str" cm="1">
-        <f t="array" ref="B5">_xll.qlFlatForward($B$2,0.03)</f>
+      <c r="B5" s="2" t="str">
+        <f>_xll.qlFlatForward($B$2,0.03,"actual365fixed")</f>
         <v>欣[test_alias_repository.xlsx]Ibor Leg!R5C2YieldTermStructureHandle,A</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -563,25 +552,34 @@
         <v>DISC_CURVE#0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="2" t="str" cm="1">
         <f t="array" ref="B8">_xll.qlAliasSet("Proj_Curve",B5)</f>
-        <v>PROJ_CURVE#0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+        <v xml:space="preserve">TypeError: TypeError: Alias PROJ_CURVE already exists with current type: &lt;class 'str'&gt;. Cannot update with new type: &lt;class 'QuantLib.QuantLib.YieldTermStructureHandle'&gt;. Delete the existing alias first or use a different alias.
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\extras\alias_repository.py", line 148, in qlAliasSet
+    return _set(alias, obj)
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\extras\alias_repository.py", line 61, in _set
+    raise TypeError(
+    ...&lt;3 lines&gt;...
+    )
+TypeError: Alias PROJ_CURVE already exists with current type: &lt;class 'str'&gt;. Cannot update with new type: &lt;class 'QuantLib.QuantLib.YieldTermStructureHandle'&gt;. Delete the existing alias first or use a different alias.
+</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="2" t="str" cm="1">
         <f t="array" ref="B10">_xll.qlAliasSet("Euribor3m",_xll.qlEuribor("3m",_xll.qlAliasGet("Proj_Curve"),B8))</f>
-        <v>EURIBOR3M#0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+        <v>EURIBOR3M#2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -590,7 +588,7 @@
         <v>46176</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -599,7 +597,7 @@
         <v>46541</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -608,7 +606,7 @@
         <v>SCHEDULE#0</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -616,7 +614,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -625,7 +623,7 @@
         <v>SCHEDULE#0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -633,25 +631,81 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>13</v>
       </c>
       <c r="B19" s="2" t="str" cm="1">
         <f t="array" ref="B19">_xll.qlAliasSet("IborLeg",_xll.qlIborLeg(B16,_xll.qlAliasGet(B17),_xll.qlAliasGet(B18),,,,,,,,,B10))</f>
-        <v>IBORLEG#0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+        <v>IBORLEG#1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
       <c r="A21" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="2" cm="1">
+      <c r="B21" s="2" t="str" cm="1">
         <f t="array" ref="B21">_xll.qlCashFlowsNpv(_xll.qlAliasGet(B19),_xll.qlAliasGet("Disc_Curve"),FALSE,,,B7:B8)</f>
-        <v>291.44819423660084</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+        <v xml:space="preserve">TypeError: TypeError: Wrong number or type of arguments for overloaded function 'CashFlows_npv'.
+  Possible C/C++ prototypes are:
+    CashFlows::npv(Leg const &amp;,YieldTermStructure const &amp;,bool,Date const &amp;,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,YieldTermStructure const &amp;,bool,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,YieldTermStructure const &amp;,bool)
+    CashFlows::npv(Leg const &amp;,Handle&lt; YieldTermStructure &gt; const &amp;,bool,Date const &amp;,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,Handle&lt; YieldTermStructure &gt; const &amp;,bool,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,Handle&lt; YieldTermStructure &gt; const &amp;,bool)
+    CashFlows::npv(Leg const &amp;,InterestRate const &amp;,bool,Date,Date)
+    CashFlows::npv(Leg const &amp;,InterestRate const &amp;,bool,Date)
+    CashFlows::npv(Leg const &amp;,InterestRate const &amp;,bool)
+    CashFlows::npv(Leg const &amp;,Rate,DayCounter const &amp;,Compounding,Frequency,bool,Date,Date)
+    CashFlows::npv(Leg const &amp;,Rate,DayCounter const &amp;,Compounding,Frequency,bool,Date)
+    CashFlows::npv(Leg const &amp;,Rate,DayCounter const &amp;,Compounding,Frequency,bool)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,Compounding,Frequency,ext::optional&lt; bool &gt;,Date const &amp;,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,Compounding,Frequency,ext::optional&lt; bool &gt;,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,Compounding,Frequency,ext::optional&lt; bool &gt;)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,Compounding,Frequency)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,DayCounter const &amp;,Compounding,Frequency,bool,Date const &amp;,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,DayCounter const &amp;,Compounding,Frequency,bool,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,DayCounter const &amp;,Compounding,Frequency,bool)
+Traceback (most recent call last):
+  File "C:\Users\kerst\Desktop\FRAME\Pricing Software\Quantlib\QuantLibXlOil\src\quantlib_xloil\cashflows.py", line 2391, in qlCashFlowsNpv
+    return ql.CashFlows.npv(
+           ~~~~~~~~~~~~~~~~^
+        to_object_list(leg, ql.CashFlow),
+        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+    ...&lt;3 lines&gt;...
+        npv_date,
+        ^^^^^^^^^
+    )
+    ^
+  File "C:\Users\kerst\.conda\envs\qlxloil\Lib\site-packages\QuantLib\QuantLib.py", line 15299, in npv
+    return _QuantLib.CashFlows_npv(*args)
+           ~~~~~~~~~~~~~~~~~~~~~~~^^^^^^^
+TypeError: Wrong number or type of arguments for overloaded function 'CashFlows_npv'.
+  Possible C/C++ prototypes are:
+    CashFlows::npv(Leg const &amp;,YieldTermStructure const &amp;,bool,Date const &amp;,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,YieldTermStructure const &amp;,bool,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,YieldTermStructure const &amp;,bool)
+    CashFlows::npv(Leg const &amp;,Handle&lt; YieldTermStructure &gt; const &amp;,bool,Date const &amp;,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,Handle&lt; YieldTermStructure &gt; const &amp;,bool,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,Handle&lt; YieldTermStructure &gt; const &amp;,bool)
+    CashFlows::npv(Leg const &amp;,InterestRate const &amp;,bool,Date,Date)
+    CashFlows::npv(Leg const &amp;,InterestRate const &amp;,bool,Date)
+    CashFlows::npv(Leg const &amp;,InterestRate const &amp;,bool)
+    CashFlows::npv(Leg const &amp;,Rate,DayCounter const &amp;,Compounding,Frequency,bool,Date,Date)
+    CashFlows::npv(Leg const &amp;,Rate,DayCounter const &amp;,Compounding,Frequency,bool,Date)
+    CashFlows::npv(Leg const &amp;,Rate,DayCounter const &amp;,Compounding,Frequency,bool)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,Compounding,Frequency,ext::optional&lt; bool &gt;,Date const &amp;,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,Compounding,Frequency,ext::optional&lt; bool &gt;,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,Compounding,Frequency,ext::optional&lt; bool &gt;)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,Compounding,Frequency)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,DayCounter const &amp;,Compounding,Frequency,bool,Date const &amp;,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,DayCounter const &amp;,Compounding,Frequency,bool,Date const &amp;)
+    CashFlows::npv(Leg const &amp;,ext::shared_ptr&lt; YieldTermStructure &gt; const &amp;,Spread,DayCounter const &amp;,Compounding,Frequency,bool)
+</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>15</v>
       </c>
@@ -660,7 +714,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2">
       <c r="B25" s="6"/>
     </row>
   </sheetData>
@@ -671,19 +725,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F54CECCD-0510-486C-9A1F-B00724C98487}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" customWidth="1"/>
-    <col min="2" max="2" width="72.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="21.77734375" customWidth="1"/>
+    <col min="1" max="1" width="19.625" customWidth="1"/>
+    <col min="2" max="2" width="72.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="21.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15">
       <c r="A1" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2" t="str" cm="1">
         <f t="array" ref="A2:E7">_xll.qlAliasGetRepository('Ibor Leg'!B21)</f>
         <v>ALIAS</v>
@@ -701,135 +755,135 @@
         <v>UPDATED</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3" t="str">
-        <v>PROJ_CURVE</v>
+        <v>DISC_CURVE</v>
       </c>
       <c r="B3" t="str">
-        <v>欣[test_alias_repository.xlsx]Dictionary!R2C1YieldTermStructureHandle,A</v>
+        <v>欣[test_alias_repository.xlsx]Dictionary!R2C1:R7C5YieldTermStructureHandle,A</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3" s="3">
-        <v>46251.791077476519</v>
+        <v>46275.634923697617</v>
       </c>
       <c r="E3" s="3">
-        <v>46251.791077476541</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>46275.634923697937</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="str">
-        <v>DISC_CURVE</v>
+        <v>PROJ_CURVE</v>
       </c>
       <c r="B4" t="str">
-        <v>欣[test_alias_repository.xlsx]Dictionary!R2C1YieldTermStructureHandle,B</v>
+        <v>Error in arg 3 'daycounter': Cannot convert '': Custom converter failed</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4" s="3">
-        <v>46251.791077476817</v>
+        <v>46275.634923700964</v>
       </c>
       <c r="E4" s="3">
-        <v>46251.791077476817</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+        <v>46275.634923701022</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="str">
-        <v>EURIBOR3M</v>
+        <v>SCHEDULE</v>
       </c>
       <c r="B5" t="str">
-        <v>欣[test_alias_repository.xlsx]Dictionary!R2C1Euribor,A</v>
+        <v>欣[test_alias_repository.xlsx]Dictionary!R2C1:R7C5Schedule,A</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5" s="3">
-        <v>46251.791077482405</v>
+        <v>46275.634923710139</v>
       </c>
       <c r="E5" s="3">
-        <v>46251.791077482419</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>46275.634923710175</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="str">
-        <v>SCHEDULE</v>
+        <v>EURIBOR3M</v>
       </c>
       <c r="B6" t="str">
-        <v>欣[test_alias_repository.xlsx]Dictionary!R2C1Schedule,A</v>
+        <v>Error in arg 2 'projection_curve': Cannot convert 'Error in arg 3 'daycounter': Cannot convert '': Custom converter failed': Expected cache string</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D6" s="3">
-        <v>46251.791077485206</v>
+        <v>46275.634923715217</v>
       </c>
       <c r="E6" s="3">
-        <v>46251.791077485221</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+        <v>46275.63497131515</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" t="str">
         <v>IBORLEG</v>
       </c>
       <c r="B7" t="str">
-        <v>欣[test_alias_repository.xlsx]Dictionary!R2C1numpy.ndarray,A</v>
+        <v>Error in arg 3 'index': Cannot convert 'Error in arg 2 'projection_curve': Cannot convert 'Error in arg 3 'daycounter': Cannot convert '': Custom converter failed': Expected cache string': Expected cache string</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" s="3">
-        <v>46251.791077498507</v>
+        <v>46275.634923722893</v>
       </c>
       <c r="E7" s="3">
-        <v>46251.79107749855</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+        <v>46275.63497132546</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15">
       <c r="A10" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5">
       <c r="A11" t="str" cm="1">
         <f t="array" ref="A11:B15">_xll.qlAliasEnvelope(A6,A2)</f>
         <v>ALIAS</v>
       </c>
       <c r="B11" s="2" t="str">
-        <v>SCHEDULE</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+        <v>EURIBOR3M</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12" t="str">
         <v>OBJECT</v>
       </c>
       <c r="B12" s="2" t="str">
-        <v>欣[test_alias_repository.xlsx]Dictionary!R11C1Schedule,A</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+        <v>Error in arg 2 'projection_curve': Cannot convert 'Error in arg 3 'daycounter': Cannot convert '': Custom converter failed': Expected cache string</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
       <c r="A13" t="str">
         <v>VERSION</v>
       </c>
       <c r="B13" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
       <c r="A14" t="str">
         <v>CREATED</v>
       </c>
       <c r="B14" s="3">
-        <v>46251.791077485206</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+        <v>46275.634923715217</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
       <c r="A15" t="str">
         <v>UPDATED</v>
       </c>
       <c r="B15" s="3">
-        <v>46251.791077485221</v>
+        <v>46275.63497131515</v>
       </c>
     </row>
   </sheetData>

</xml_diff>